<commit_message>
Auto Update Lottery Data
</commit_message>
<xml_diff>
--- a/最新開獎紀錄.xlsx
+++ b/最新開獎紀錄.xlsx
@@ -968,151 +968,151 @@
     </row>
     <row r="2" ht="20" customHeight="1" s="5">
       <c r="A2" s="4" t="n">
-        <v>115000207</v>
+        <v>115000208</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>115.08.26</t>
+          <t>115.08.27</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>13  19  23  35  38</t>
+          <t>02  03  07  25  33</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" s="5">
       <c r="A3" s="4" t="n">
-        <v>115000208</v>
+        <v>115000209</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>115.08.27</t>
+          <t>115.08.28</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>02  03  07  25  33</t>
+          <t>02  04  09  12  36</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" s="5">
       <c r="A4" s="4" t="n">
-        <v>115000209</v>
+        <v>115000210</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>115.08.28</t>
+          <t>115.08.29</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>02  04  09  12  36</t>
+          <t>03  06  17  23  33</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" s="5">
       <c r="A5" s="4" t="n">
-        <v>115000210</v>
+        <v>115000211</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>115.08.29</t>
+          <t>115.08.31</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>03  06  17  23  33</t>
+          <t>05  10  12  33  39</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" s="5">
       <c r="A6" s="4" t="n">
-        <v>115000211</v>
+        <v>115000212</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>115.08.31</t>
+          <t>115.09.01</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>05  10  12  33  39</t>
+          <t>02  04  22  30  38</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" s="5">
       <c r="A7" s="4" t="n">
-        <v>115000212</v>
+        <v>115000213</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>115.09.01</t>
+          <t>115.09.02</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>02  04  22  30  38</t>
+          <t>07  08  13  16  18</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" s="5">
       <c r="A8" s="4" t="n">
-        <v>115000213</v>
+        <v>115000214</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>115.09.02</t>
+          <t>115.09.03</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>07  08  13  16  18</t>
+          <t>18  19  22  23  34</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" s="5">
       <c r="A9" s="4" t="n">
-        <v>115000214</v>
+        <v>115000215</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>115.09.03</t>
+          <t>115.09.04</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>18  19  22  23  34</t>
+          <t>02  04  15  17  24</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" s="5">
       <c r="A10" s="4" t="n">
-        <v>115000215</v>
+        <v>115000216</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>115.09.04</t>
+          <t>115.09.05</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>02  04  15  17  24</t>
+          <t>03  08  10  28  38</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" s="5">
       <c r="A11" s="4" t="n">
-        <v>115000216</v>
+        <v>115000217</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>115.09.05</t>
+          <t>115.09.07</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>03  08  10  28  38</t>
+          <t>19  25  26  31  35</t>
         </is>
       </c>
     </row>
@@ -1354,201 +1354,201 @@
     </row>
     <row r="2" ht="20" customHeight="1" s="5">
       <c r="A2" s="4" t="n">
-        <v>115000062</v>
+        <v>115000063</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>115.08.03</t>
+          <t>115.08.06</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>04  15  22  26  34  36</t>
+          <t>02  07  08  20  26  33</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>04</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" s="5">
       <c r="A3" s="4" t="n">
-        <v>115000063</v>
+        <v>115000064</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>115.08.06</t>
+          <t>115.08.10</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>02  07  08  20  26  33</t>
+          <t>11  25  28  30  31  36</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" s="5">
       <c r="A4" s="4" t="n">
-        <v>115000064</v>
+        <v>115000065</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>115.08.10</t>
+          <t>115.08.13</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>11  25  28  30  31  36</t>
+          <t>01  03  04  07  10  19</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>06</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" s="5">
       <c r="A5" s="4" t="n">
-        <v>115000065</v>
+        <v>115000066</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>115.08.13</t>
+          <t>115.08.17</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>01  03  04  07  10  19</t>
+          <t>05  11  18  19  35  38</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>08</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" s="5">
       <c r="A6" s="4" t="n">
-        <v>115000066</v>
+        <v>115000067</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>115.08.17</t>
+          <t>115.08.20</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>05  11  18  19  35  38</t>
+          <t>01  02  09  11  29  35</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>02</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" s="5">
       <c r="A7" s="4" t="n">
-        <v>115000067</v>
+        <v>115000068</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>115.08.20</t>
+          <t>115.08.24</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>01  02  09  11  29  35</t>
+          <t>06  07  09  23  26  36</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>07</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" s="5">
       <c r="A8" s="4" t="n">
-        <v>115000068</v>
+        <v>115000069</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>115.08.24</t>
+          <t>115.08.27</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>06  07  09  23  26  36</t>
+          <t>02  07  09  11  24  36</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>01</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" s="5">
       <c r="A9" s="4" t="n">
-        <v>115000069</v>
+        <v>115000070</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>115.08.27</t>
+          <t>115.08.31</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>02  07  09  11  24  36</t>
+          <t>04  08  12  19  32  37</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" s="5">
       <c r="A10" s="4" t="n">
-        <v>115000070</v>
+        <v>115000071</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>115.08.31</t>
+          <t>115.09.03</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>04  08  12  19  32  37</t>
+          <t>01  06  07  19  30  33</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>08</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" s="5">
       <c r="A11" s="4" t="n">
-        <v>115000071</v>
+        <v>115000072</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>115.09.03</t>
+          <t>115.09.07</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>01  06  07  19  30  33</t>
+          <t>07  14  17  22  29  35</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>02</t>
         </is>
       </c>
     </row>

</xml_diff>